<commit_message>
Use generic domain example naming
</commit_message>
<xml_diff>
--- a/demo_data/harbor_job/forecast-update__trial-017/artifacts/workspace/forecast.xlsx
+++ b/demo_data/harbor_job/forecast-update__trial-017/artifacts/workspace/forecast.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb0d84d9506eb4101"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rcb202e0ca12749cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="Raaa6ca4c343f4d71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="4" r:id="Re24185347d7e4071"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6a7a4ebfad6c4f04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rc381a7ad21494d07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="Rd54dafe8008f4110"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="4" r:id="R1e6ec0614ecb43dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -666,7 +666,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9974453f9d9e4e5a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R547389ac135e4946"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -893,28 +893,28 @@
     </x:row>
     <x:row r="3" ht="21" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Illustrative artifact used in the Acto × Harbor × marimo integration demo</x:v>
+        <x:v>Illustrative artifact used in the Harbor + Marimo domain example</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>Illustrative artifact used in the Acto × Harbor × marimo integration demo</x:v>
+        <x:v>Illustrative artifact used in the Harbor + Marimo domain example</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Illustrative artifact used in the Acto × Harbor × marimo integration demo</x:v>
+        <x:v>Illustrative artifact used in the Harbor + Marimo domain example</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Illustrative artifact used in the Acto × Harbor × marimo integration demo</x:v>
+        <x:v>Illustrative artifact used in the Harbor + Marimo domain example</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Illustrative artifact used in the Acto × Harbor × marimo integration demo</x:v>
+        <x:v>Illustrative artifact used in the Harbor + Marimo domain example</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Illustrative artifact used in the Acto × Harbor × marimo integration demo</x:v>
+        <x:v>Illustrative artifact used in the Harbor + Marimo domain example</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Illustrative artifact used in the Acto × Harbor × marimo integration demo</x:v>
+        <x:v>Illustrative artifact used in the Harbor + Marimo domain example</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str">
-        <x:v>Illustrative artifact used in the Acto × Harbor × marimo integration demo</x:v>
+        <x:v>Illustrative artifact used in the Harbor + Marimo domain example</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1072,7 +1072,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="63" t="str">
-        <x:v>This is a synthetic workbook used to make Harbor's artifact handoff visible. The case study is about the integration pattern, not the finance example.</x:v>
+        <x:v>Synthetic workbook used to demonstrate Harbor artifact analysis.</x:v>
       </x:c>
       <x:c r="B22" s="63"/>
       <x:c r="C22" s="63"/>
@@ -1084,7 +1084,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="63" t="str">
-        <x:v>Open the Forecast sheet to inspect the underlying formulas and assumptions.</x:v>
+        <x:v>Open the Forecast sheet to inspect formulas and assumptions.</x:v>
       </x:c>
       <x:c r="B23" s="63"/>
       <x:c r="C23" s="63"/>
@@ -1109,7 +1109,7 @@
     <x:mergeCell ref="A23:H23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c0dec10e2ba49f2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8135ba6a9af248a1"/>
 </x:worksheet>
 </file>
 

</xml_diff>